<commit_message>
Add Track B module B12 School Operations and 30 school data elements
- B12 (13 questions, drafted by DUATF): parental consent, admission data and notice,
  tracking and monitoring within the Fourth Schedule, no advertising or detrimental use,
  transport, health and child-protection records, photos, sharing, retention, parents'
  rights, visitors and learning platforms. Each lists the evidence to ask for and maps to
  the children's obligations; questions on children's duties carry High risk.
- 30 data elements for schools (admissions, report cards, transfer certificates, special
  needs plans, UDISE+ PEN, RTE category proof, bus routes and GPS, medical room records,
  POCSO records, classroom CCTV, student photos, fees, parent communications and more),
  and a "School operations" suggestion preset.
- 201 questions and 212 data elements in all. Plan C20.10 with its test; ADR-0007.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seed/question-bank/source/TPL-002_Internal_Data_Handlers.xlsx
+++ b/seed/question-bank/source/TPL-002_Internal_Data_Handlers.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="403">
   <si>
     <t>Question ID</t>
   </si>
@@ -1026,6 +1026,229 @@
 Backup and data retention handling procedure
 Final access review
 Sample completed vendor offboarding record</t>
+  </si>
+  <si>
+    <t>c0000001-bc00-0000-0000-000000000001</t>
+  </si>
+  <si>
+    <t>School Operations</t>
+  </si>
+  <si>
+    <t>B12.1</t>
+  </si>
+  <si>
+    <t>Is a parent's or lawful guardian's verifiable consent obtained before a student's personal data is processed on the basis of consent?</t>
+  </si>
+  <si>
+    <t>HIGH</t>
+  </si>
+  <si>
+    <t>S.9(1), Rule 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admission form with the parental consent section
+Consent records for each student
+How the school checks that the person consenting is the parent or guardian and an adult</t>
+  </si>
+  <si>
+    <t>c0000002-bc00-0000-0000-000000000001</t>
+  </si>
+  <si>
+    <t>B12.2</t>
+  </si>
+  <si>
+    <t>Does the admission process collect only the student and parent data the school needs, with a notice that lists that data and its purposes?</t>
+  </si>
+  <si>
+    <t>MEDIUM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admission form
+Privacy notice for parents
+List of admission data fields with the purpose of each</t>
+  </si>
+  <si>
+    <t>c0000003-bc00-0000-0000-000000000001</t>
+  </si>
+  <si>
+    <t>B12.3</t>
+  </si>
+  <si>
+    <t>Is tracking or behavioural monitoring of students (classroom CCTV, bus GPS, attendance or learning apps) limited to educational activities and student safety?</t>
+  </si>
+  <si>
+    <t>S.9(3), S.9(4), Rule 12, Fourth Schedule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">List of monitoring and tracking in use, with the purpose of each
+CCTV and GPS policy
+Exemption register entry for each Fourth Schedule purpose relied on</t>
+  </si>
+  <si>
+    <t>c0000004-bc00-0000-0000-000000000001</t>
+  </si>
+  <si>
+    <t>B12.4</t>
+  </si>
+  <si>
+    <t>Are students' data kept from advertising, marketing and any use detrimental to their well-being, including promotions by ed-tech, uniform or book vendors?</t>
+  </si>
+  <si>
+    <t>S.9(2), S.9(3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Policy on use of student data
+Vendor contracts with no-marketing clauses
+Declaration of no targeted advertising to students</t>
+  </si>
+  <si>
+    <t>c0000005-bc00-0000-0000-000000000001</t>
+  </si>
+  <si>
+    <t>B12.5</t>
+  </si>
+  <si>
+    <t>Is school transport data (routes, stops, pick-up times, GPS tracking, driver and attendant details) access-controlled and shared only with parents and authorised staff?</t>
+  </si>
+  <si>
+    <t>S.8(5), Rule 6, Fourth Schedule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transport app access list
+Transport vendor contract
+Driver and attendant verification records</t>
+  </si>
+  <si>
+    <t>c0000006-bc00-0000-0000-000000000001</t>
+  </si>
+  <si>
+    <t>B12.6</t>
+  </si>
+  <si>
+    <t>Are students' health records (medical room visits, allergies, vaccinations, special needs) kept confidential and open only to the staff who need them?</t>
+  </si>
+  <si>
+    <t>S.8(5), Rule 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medical room register and where it is kept
+Access list for health records
+Procedure for sharing health information with teachers</t>
+  </si>
+  <si>
+    <t>c0000007-bc00-0000-0000-000000000001</t>
+  </si>
+  <si>
+    <t>B12.7</t>
+  </si>
+  <si>
+    <t>Are counselling, disciplinary and child-protection (POCSO) records kept separately, with access restricted to the designated staff?</t>
+  </si>
+  <si>
+    <t>S.8(5), S.9(2), Rule 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Child protection policy
+Access list for counselling and incident records
+Storage arrangement for these records</t>
+  </si>
+  <si>
+    <t>c0000008-bc00-0000-0000-000000000001</t>
+  </si>
+  <si>
+    <t>B12.8</t>
+  </si>
+  <si>
+    <t>Are photos and videos of students published (website, social media, newsletters) only with parental consent, and taken down when consent is withdrawn?</t>
+  </si>
+  <si>
+    <t>S.6(4), S.9(1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Photo and video consent form
+Register of consents and withdrawals
+Take-down procedure</t>
+  </si>
+  <si>
+    <t>c0000009-bc00-0000-0000-000000000001</t>
+  </si>
+  <si>
+    <t>B12.9</t>
+  </si>
+  <si>
+    <t>Are student and parent records shared with boards, government portals and ed-tech or transport vendors only where a law requires it or under a contract?</t>
+  </si>
+  <si>
+    <t>S.7, S.8(2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">List of portals and vendors that receive student data, with the legal basis or contract for each
+Data processing agreements with vendors</t>
+  </si>
+  <si>
+    <t>c0000010-bc00-0000-0000-000000000001</t>
+  </si>
+  <si>
+    <t>B12.10</t>
+  </si>
+  <si>
+    <t>Is there a retention schedule for admission, academic, fee and transfer records, including applicants not admitted and students who have left?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retention schedule for student records
+Deletion or archival log
+Board or regulatory retention requirements relied on</t>
+  </si>
+  <si>
+    <t>c0000011-bc00-0000-0000-000000000001</t>
+  </si>
+  <si>
+    <t>B12.11</t>
+  </si>
+  <si>
+    <t>Can parents ask to see, correct or erase their child's data and raise grievances, and does the school verify that the request comes from the parent or guardian?</t>
+  </si>
+  <si>
+    <t>S.11-S.13, Rule 14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rights request form or channel for parents
+Requester verification procedure
+Rights and grievance request log</t>
+  </si>
+  <si>
+    <t>c0000012-bc00-0000-0000-000000000001</t>
+  </si>
+  <si>
+    <t>B12.12</t>
+  </si>
+  <si>
+    <t>Are visitor, gate-pass and authorised pick-up records controlled and kept only as long as they are needed?</t>
+  </si>
+  <si>
+    <t>S.8(5), S.8(7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visitor and gate-pass register
+Authorised pick-up list procedure
+Retention period for these records</t>
+  </si>
+  <si>
+    <t>c0000013-bc00-0000-0000-000000000001</t>
+  </si>
+  <si>
+    <t>B12.13</t>
+  </si>
+  <si>
+    <t>Are student accounts on learning platforms and school apps set up without behavioural profiling or targeted advertising, and are the vendor terms checked for this?</t>
+  </si>
+  <si>
+    <t>S.9(3), S.8(2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">List of learning platforms and apps with student accounts
+Vendor terms or data processing agreements
+Platform privacy settings for students</t>
   </si>
   <si>
     <t>Consent</t>
@@ -1474,7 +1697,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -3441,8 +3664,424 @@
         <v>313</v>
       </c>
     </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>314</v>
+      </c>
+      <c r="B62" t="s">
+        <v>315</v>
+      </c>
+      <c r="C62" t="s">
+        <v>316</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="E62" t="s">
+        <v>46</v>
+      </c>
+      <c r="F62" t="s">
+        <v>24</v>
+      </c>
+      <c r="G62" t="s">
+        <v>318</v>
+      </c>
+      <c r="H62" t="s">
+        <v>319</v>
+      </c>
+      <c r="I62" t="s">
+        <v>18</v>
+      </c>
+      <c r="J62" s="1" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>321</v>
+      </c>
+      <c r="B63" t="s">
+        <v>315</v>
+      </c>
+      <c r="C63" t="s">
+        <v>322</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="E63" t="s">
+        <v>40</v>
+      </c>
+      <c r="F63" t="s">
+        <v>24</v>
+      </c>
+      <c r="G63" t="s">
+        <v>324</v>
+      </c>
+      <c r="H63" t="s">
+        <v>268</v>
+      </c>
+      <c r="I63" t="s">
+        <v>18</v>
+      </c>
+      <c r="J63" s="1" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>326</v>
+      </c>
+      <c r="B64" t="s">
+        <v>315</v>
+      </c>
+      <c r="C64" t="s">
+        <v>327</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="E64" t="s">
+        <v>40</v>
+      </c>
+      <c r="F64" t="s">
+        <v>24</v>
+      </c>
+      <c r="G64" t="s">
+        <v>318</v>
+      </c>
+      <c r="H64" t="s">
+        <v>329</v>
+      </c>
+      <c r="I64" t="s">
+        <v>18</v>
+      </c>
+      <c r="J64" s="1" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>331</v>
+      </c>
+      <c r="B65" t="s">
+        <v>315</v>
+      </c>
+      <c r="C65" t="s">
+        <v>332</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="E65" t="s">
+        <v>46</v>
+      </c>
+      <c r="F65" t="s">
+        <v>24</v>
+      </c>
+      <c r="G65" t="s">
+        <v>318</v>
+      </c>
+      <c r="H65" t="s">
+        <v>334</v>
+      </c>
+      <c r="I65" t="s">
+        <v>18</v>
+      </c>
+      <c r="J65" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>336</v>
+      </c>
+      <c r="B66" t="s">
+        <v>315</v>
+      </c>
+      <c r="C66" t="s">
+        <v>337</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="E66" t="s">
+        <v>40</v>
+      </c>
+      <c r="F66" t="s">
+        <v>24</v>
+      </c>
+      <c r="G66" t="s">
+        <v>324</v>
+      </c>
+      <c r="H66" t="s">
+        <v>339</v>
+      </c>
+      <c r="I66" t="s">
+        <v>18</v>
+      </c>
+      <c r="J66" s="1" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>341</v>
+      </c>
+      <c r="B67" t="s">
+        <v>315</v>
+      </c>
+      <c r="C67" t="s">
+        <v>342</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="E67" t="s">
+        <v>40</v>
+      </c>
+      <c r="F67" t="s">
+        <v>24</v>
+      </c>
+      <c r="G67" t="s">
+        <v>324</v>
+      </c>
+      <c r="H67" t="s">
+        <v>344</v>
+      </c>
+      <c r="I67" t="s">
+        <v>18</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>346</v>
+      </c>
+      <c r="B68" t="s">
+        <v>315</v>
+      </c>
+      <c r="C68" t="s">
+        <v>347</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="E68" t="s">
+        <v>40</v>
+      </c>
+      <c r="F68" t="s">
+        <v>24</v>
+      </c>
+      <c r="G68" t="s">
+        <v>318</v>
+      </c>
+      <c r="H68" t="s">
+        <v>349</v>
+      </c>
+      <c r="I68" t="s">
+        <v>18</v>
+      </c>
+      <c r="J68" s="1" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>351</v>
+      </c>
+      <c r="B69" t="s">
+        <v>315</v>
+      </c>
+      <c r="C69" t="s">
+        <v>352</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E69" t="s">
+        <v>46</v>
+      </c>
+      <c r="F69" t="s">
+        <v>24</v>
+      </c>
+      <c r="G69" t="s">
+        <v>324</v>
+      </c>
+      <c r="H69" t="s">
+        <v>354</v>
+      </c>
+      <c r="I69" t="s">
+        <v>18</v>
+      </c>
+      <c r="J69" s="1" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>356</v>
+      </c>
+      <c r="B70" t="s">
+        <v>315</v>
+      </c>
+      <c r="C70" t="s">
+        <v>357</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="E70" t="s">
+        <v>46</v>
+      </c>
+      <c r="F70" t="s">
+        <v>24</v>
+      </c>
+      <c r="G70" t="s">
+        <v>324</v>
+      </c>
+      <c r="H70" t="s">
+        <v>359</v>
+      </c>
+      <c r="I70" t="s">
+        <v>18</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>361</v>
+      </c>
+      <c r="B71" t="s">
+        <v>315</v>
+      </c>
+      <c r="C71" t="s">
+        <v>362</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="E71" t="s">
+        <v>40</v>
+      </c>
+      <c r="F71" t="s">
+        <v>24</v>
+      </c>
+      <c r="G71" t="s">
+        <v>324</v>
+      </c>
+      <c r="H71" t="s">
+        <v>88</v>
+      </c>
+      <c r="I71" t="s">
+        <v>18</v>
+      </c>
+      <c r="J71" s="1" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>365</v>
+      </c>
+      <c r="B72" t="s">
+        <v>315</v>
+      </c>
+      <c r="C72" t="s">
+        <v>366</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E72" t="s">
+        <v>40</v>
+      </c>
+      <c r="F72" t="s">
+        <v>24</v>
+      </c>
+      <c r="G72" t="s">
+        <v>324</v>
+      </c>
+      <c r="H72" t="s">
+        <v>368</v>
+      </c>
+      <c r="I72" t="s">
+        <v>18</v>
+      </c>
+      <c r="J72" s="1" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>370</v>
+      </c>
+      <c r="B73" t="s">
+        <v>315</v>
+      </c>
+      <c r="C73" t="s">
+        <v>371</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="E73" t="s">
+        <v>40</v>
+      </c>
+      <c r="F73" t="s">
+        <v>24</v>
+      </c>
+      <c r="G73" t="s">
+        <v>16</v>
+      </c>
+      <c r="H73" t="s">
+        <v>373</v>
+      </c>
+      <c r="I73" t="s">
+        <v>18</v>
+      </c>
+      <c r="J73" s="1" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>375</v>
+      </c>
+      <c r="B74" t="s">
+        <v>315</v>
+      </c>
+      <c r="C74" t="s">
+        <v>376</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="E74" t="s">
+        <v>46</v>
+      </c>
+      <c r="F74" t="s">
+        <v>24</v>
+      </c>
+      <c r="G74" t="s">
+        <v>318</v>
+      </c>
+      <c r="H74" t="s">
+        <v>378</v>
+      </c>
+      <c r="I74" t="s">
+        <v>18</v>
+      </c>
+      <c r="J74" s="1" t="s">
+        <v>379</v>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="54">
+  <dataValidations count="67">
     <dataValidation type="list" allowBlank="1" sqref="F10">
       <formula1>_options!$A$10:$E$10</formula1>
     </dataValidation>
@@ -3599,8 +4238,47 @@
     <dataValidation type="list" allowBlank="1" sqref="F61">
       <formula1>_options!$A$61:$E$61</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F62">
+      <formula1>_options!$A$62:$D$62</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F63">
+      <formula1>_options!$A$63:$E$63</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F64">
+      <formula1>_options!$A$64:$E$64</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F65">
+      <formula1>_options!$A$65:$D$65</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F66">
+      <formula1>_options!$A$66:$E$66</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F67">
+      <formula1>_options!$A$67:$E$67</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F68">
+      <formula1>_options!$A$68:$E$68</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F69">
+      <formula1>_options!$A$69:$D$69</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="F7">
       <formula1>_options!$A$7:$D$7</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F70">
+      <formula1>_options!$A$70:$D$70</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F71">
+      <formula1>_options!$A$71:$E$71</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F72">
+      <formula1>_options!$A$72:$E$72</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F73">
+      <formula1>_options!$A$73:$E$73</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F74">
+      <formula1>_options!$A$74:$D$74</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="F8">
       <formula1>_options!$A$8:$D$8</formula1>
@@ -3613,480 +4291,480 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:F61"/>
+  <dimension ref="A3:F74"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>314</v>
+        <v>380</v>
       </c>
       <c r="B3" t="s">
-        <v>315</v>
+        <v>381</v>
       </c>
       <c r="C3" t="s">
-        <v>316</v>
+        <v>382</v>
       </c>
       <c r="D3" t="s">
-        <v>317</v>
+        <v>383</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>318</v>
+        <v>384</v>
       </c>
       <c r="B5" t="s">
-        <v>319</v>
+        <v>385</v>
       </c>
       <c r="C5" t="s">
-        <v>320</v>
+        <v>386</v>
       </c>
       <c r="D5" t="s">
-        <v>321</v>
+        <v>387</v>
       </c>
       <c r="E5" t="s">
-        <v>322</v>
+        <v>388</v>
       </c>
       <c r="F5" t="s">
-        <v>323</v>
+        <v>389</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B6" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C6" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D6" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E6" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B7" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C7" t="s">
         <v>18</v>
       </c>
       <c r="D7" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B8" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C8" t="s">
         <v>18</v>
       </c>
       <c r="D8" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B10" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C10" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D10" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E10" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B11" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C11" t="s">
         <v>18</v>
       </c>
       <c r="D11" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B12" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C12" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D12" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E12" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B13" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C13" t="s">
         <v>18</v>
       </c>
       <c r="D13" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B14" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C14" t="s">
         <v>18</v>
       </c>
       <c r="D14" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B15" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C15" t="s">
         <v>18</v>
       </c>
       <c r="D15" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B16" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C16" t="s">
         <v>18</v>
       </c>
       <c r="D16" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B17" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C17" t="s">
         <v>18</v>
       </c>
       <c r="D17" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B18" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C18" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D18" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E18" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B19" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C19" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D19" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E19" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B20" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C20" t="s">
         <v>18</v>
       </c>
       <c r="D20" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B21" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C21" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D21" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E21" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B22" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C22" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D22" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E22" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B23" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C23" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D23" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E23" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B24" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C24" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D24" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E24" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B25" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C25" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D25" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E25" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B26" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C26" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D26" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E26" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B27" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C27" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D27" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E27" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B28" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C28" t="s">
         <v>18</v>
       </c>
       <c r="D28" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B29" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C29" t="s">
         <v>18</v>
       </c>
       <c r="D29" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B30" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C30" t="s">
         <v>18</v>
       </c>
       <c r="D30" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B32" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C32" t="s">
         <v>18</v>
       </c>
       <c r="D32" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B33" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C33" t="s">
         <v>18</v>
       </c>
       <c r="D33" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>332</v>
+        <v>398</v>
       </c>
       <c r="B34" t="s">
-        <v>333</v>
+        <v>399</v>
       </c>
       <c r="C34" t="s">
-        <v>334</v>
+        <v>400</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B35" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C35" t="s">
         <v>18</v>
       </c>
       <c r="D35" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B36" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C36" t="s">
         <v>18</v>
       </c>
       <c r="D36" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -4094,363 +4772,569 @@
         <v>18</v>
       </c>
       <c r="B37" t="s">
-        <v>335</v>
+        <v>401</v>
       </c>
       <c r="C37" t="s">
-        <v>336</v>
+        <v>402</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B38" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C38" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D38" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E38" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B40" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C40" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D40" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E40" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B41" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C41" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D41" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E41" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B42" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C42" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D42" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E42" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B43" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C43" t="s">
         <v>18</v>
       </c>
       <c r="D43" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B44" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C44" t="s">
         <v>18</v>
       </c>
       <c r="D44" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B45" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C45" t="s">
         <v>18</v>
       </c>
       <c r="D45" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B46" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C46" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D46" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E46" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B47" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C47" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D47" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E47" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B48" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C48" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D48" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E48" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B49" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C49" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D49" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E49" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B50" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C50" t="s">
         <v>18</v>
       </c>
       <c r="D50" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B51" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C51" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D51" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E51" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B52" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C52" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D52" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E52" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B53" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C53" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D53" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E53" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B54" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C54" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D54" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E54" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B55" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C55" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D55" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E55" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B56" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C56" t="s">
         <v>18</v>
       </c>
       <c r="D56" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B57" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C57" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D57" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E57" t="s">
-        <v>328</v>
+        <v>394</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B59" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C59" t="s">
         <v>18</v>
       </c>
       <c r="D59" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>329</v>
+        <v>395</v>
       </c>
       <c r="B60" t="s">
-        <v>330</v>
+        <v>396</v>
       </c>
       <c r="C60" t="s">
         <v>18</v>
       </c>
       <c r="D60" t="s">
-        <v>331</v>
+        <v>397</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>324</v>
+        <v>390</v>
       </c>
       <c r="B61" t="s">
-        <v>325</v>
+        <v>391</v>
       </c>
       <c r="C61" t="s">
-        <v>326</v>
+        <v>392</v>
       </c>
       <c r="D61" t="s">
-        <v>327</v>
+        <v>393</v>
       </c>
       <c r="E61" t="s">
-        <v>328</v>
+        <v>394</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>395</v>
+      </c>
+      <c r="B62" t="s">
+        <v>396</v>
+      </c>
+      <c r="C62" t="s">
+        <v>18</v>
+      </c>
+      <c r="D62" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>390</v>
+      </c>
+      <c r="B63" t="s">
+        <v>391</v>
+      </c>
+      <c r="C63" t="s">
+        <v>392</v>
+      </c>
+      <c r="D63" t="s">
+        <v>393</v>
+      </c>
+      <c r="E63" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>390</v>
+      </c>
+      <c r="B64" t="s">
+        <v>391</v>
+      </c>
+      <c r="C64" t="s">
+        <v>392</v>
+      </c>
+      <c r="D64" t="s">
+        <v>393</v>
+      </c>
+      <c r="E64" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>395</v>
+      </c>
+      <c r="B65" t="s">
+        <v>396</v>
+      </c>
+      <c r="C65" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>390</v>
+      </c>
+      <c r="B66" t="s">
+        <v>391</v>
+      </c>
+      <c r="C66" t="s">
+        <v>392</v>
+      </c>
+      <c r="D66" t="s">
+        <v>393</v>
+      </c>
+      <c r="E66" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>390</v>
+      </c>
+      <c r="B67" t="s">
+        <v>391</v>
+      </c>
+      <c r="C67" t="s">
+        <v>392</v>
+      </c>
+      <c r="D67" t="s">
+        <v>393</v>
+      </c>
+      <c r="E67" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>390</v>
+      </c>
+      <c r="B68" t="s">
+        <v>391</v>
+      </c>
+      <c r="C68" t="s">
+        <v>392</v>
+      </c>
+      <c r="D68" t="s">
+        <v>393</v>
+      </c>
+      <c r="E68" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>395</v>
+      </c>
+      <c r="B69" t="s">
+        <v>396</v>
+      </c>
+      <c r="C69" t="s">
+        <v>18</v>
+      </c>
+      <c r="D69" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>395</v>
+      </c>
+      <c r="B70" t="s">
+        <v>396</v>
+      </c>
+      <c r="C70" t="s">
+        <v>18</v>
+      </c>
+      <c r="D70" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>390</v>
+      </c>
+      <c r="B71" t="s">
+        <v>391</v>
+      </c>
+      <c r="C71" t="s">
+        <v>392</v>
+      </c>
+      <c r="D71" t="s">
+        <v>393</v>
+      </c>
+      <c r="E71" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>390</v>
+      </c>
+      <c r="B72" t="s">
+        <v>391</v>
+      </c>
+      <c r="C72" t="s">
+        <v>392</v>
+      </c>
+      <c r="D72" t="s">
+        <v>393</v>
+      </c>
+      <c r="E72" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>390</v>
+      </c>
+      <c r="B73" t="s">
+        <v>391</v>
+      </c>
+      <c r="C73" t="s">
+        <v>392</v>
+      </c>
+      <c r="D73" t="s">
+        <v>393</v>
+      </c>
+      <c r="E73" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>395</v>
+      </c>
+      <c r="B74" t="s">
+        <v>396</v>
+      </c>
+      <c r="C74" t="s">
+        <v>18</v>
+      </c>
+      <c r="D74" t="s">
+        <v>397</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Make B12 Education Operations for every kind of educational institution
- B12 School Operations becomes Education Operations, worded for schools, colleges,
  universities, polytechnics, diploma and coaching institutes: children's duties (parental
  consent, no tracking or targeted ads) are asked about students under 18.
- Education data elements reworded for all institutions, plus university enrolment
  numbers, internships and placements, alumni, research and thesis records, and
  anti-ragging and internal complaints records (217 elements in all).
- The "Education operations" preset also matches college, university, institute,
  polytechnic, diploma, campus, registrar and placement departments.
- An AI-drafted data element nobody has reviewed yet takes corrected text on update; one a
  person reviewed or edited is left alone.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seed/question-bank/source/TPL-002_Internal_Data_Handlers.xlsx
+++ b/seed/question-bank/source/TPL-002_Internal_Data_Handlers.xlsx
@@ -1031,13 +1031,13 @@
     <t>c0000001-bc00-0000-0000-000000000001</t>
   </si>
   <si>
-    <t>School Operations</t>
+    <t>Education Operations</t>
   </si>
   <si>
     <t>B12.1</t>
   </si>
   <si>
-    <t>Is a parent's or lawful guardian's verifiable consent obtained before a student's personal data is processed on the basis of consent?</t>
+    <t>For students under 18, is a parent's or lawful guardian's verifiable consent obtained before their personal data is processed on the basis of consent?</t>
   </si>
   <si>
     <t>HIGH</t>
@@ -1047,8 +1047,8 @@
   </si>
   <si>
     <t xml:space="preserve">Admission form with the parental consent section
-Consent records for each student
-How the school checks that the person consenting is the parent or guardian and an adult</t>
+Consent records for students under 18
+How the institution checks that the person consenting is the parent or guardian and an adult</t>
   </si>
   <si>
     <t>c0000002-bc00-0000-0000-000000000001</t>
@@ -1057,7 +1057,7 @@
     <t>B12.2</t>
   </si>
   <si>
-    <t>Does the admission process collect only the student and parent data the school needs, with a notice that lists that data and its purposes?</t>
+    <t>Does the admission process collect only the student and parent data the institution needs, with a notice that lists that data and its purposes?</t>
   </si>
   <si>
     <t>MEDIUM</t>
@@ -1074,7 +1074,7 @@
     <t>B12.3</t>
   </si>
   <si>
-    <t>Is tracking or behavioural monitoring of students (classroom CCTV, bus GPS, attendance or learning apps) limited to educational activities and student safety?</t>
+    <t>Is tracking or behavioural monitoring of students under 18 (classroom CCTV, bus GPS, attendance or learning apps) limited to educational activities and their safety?</t>
   </si>
   <si>
     <t>S.9(3), S.9(4), Rule 12, Fourth Schedule</t>
@@ -1091,7 +1091,7 @@
     <t>B12.4</t>
   </si>
   <si>
-    <t>Are students' data kept from advertising, marketing and any use detrimental to their well-being, including promotions by ed-tech, uniform or book vendors?</t>
+    <t>Are students' data kept from advertising, marketing and any use detrimental to their well-being, including promotions by ed-tech, coaching, uniform or book vendors?</t>
   </si>
   <si>
     <t>S.9(2), S.9(3)</t>
@@ -1108,7 +1108,7 @@
     <t>B12.5</t>
   </si>
   <si>
-    <t>Is school transport data (routes, stops, pick-up times, GPS tracking, driver and attendant details) access-controlled and shared only with parents and authorised staff?</t>
+    <t>Is student transport data (routes, stops, pick-up times, GPS tracking, driver and attendant details) access-controlled and shared only with parents, students and authorised staff?</t>
   </si>
   <si>
     <t>S.8(5), Rule 6, Fourth Schedule</t>
@@ -1125,7 +1125,7 @@
     <t>B12.6</t>
   </si>
   <si>
-    <t>Are students' health records (medical room visits, allergies, vaccinations, special needs) kept confidential and open only to the staff who need them?</t>
+    <t>Are students' health records (medical room or health centre visits, allergies, vaccinations, special needs) kept confidential and open only to the staff who need them?</t>
   </si>
   <si>
     <t>S.8(5), Rule 6</t>
@@ -1142,7 +1142,7 @@
     <t>B12.7</t>
   </si>
   <si>
-    <t>Are counselling, disciplinary and child-protection (POCSO) records kept separately, with access restricted to the designated staff?</t>
+    <t>Are counselling, disciplinary, anti-ragging, internal complaints and child-protection (POCSO) records kept separately, with access restricted to the designated staff?</t>
   </si>
   <si>
     <t>S.8(5), S.9(2), Rule 6</t>
@@ -1159,7 +1159,7 @@
     <t>B12.8</t>
   </si>
   <si>
-    <t>Are photos and videos of students published (website, social media, newsletters) only with parental consent, and taken down when consent is withdrawn?</t>
+    <t>Are photos and videos of students published (website, social media, newsletters, brochures) only with consent (a parent or guardian for students under 18), and taken down when it is withdrawn?</t>
   </si>
   <si>
     <t>S.6(4), S.9(1)</t>
@@ -1176,7 +1176,7 @@
     <t>B12.9</t>
   </si>
   <si>
-    <t>Are student and parent records shared with boards, government portals and ed-tech or transport vendors only where a law requires it or under a contract?</t>
+    <t>Are student and parent records shared with boards, universities, regulators, government portals and ed-tech, placement or transport vendors only where a law requires it or under a contract?</t>
   </si>
   <si>
     <t>S.7, S.8(2)</t>
@@ -1192,7 +1192,7 @@
     <t>B12.10</t>
   </si>
   <si>
-    <t>Is there a retention schedule for admission, academic, fee and transfer records, including applicants not admitted and students who have left?</t>
+    <t>Is there a retention schedule for admission, academic, examination, fee and transfer records, including applicants not admitted and students who have left?</t>
   </si>
   <si>
     <t xml:space="preserve">Retention schedule for student records
@@ -1206,13 +1206,13 @@
     <t>B12.11</t>
   </si>
   <si>
-    <t>Can parents ask to see, correct or erase their child's data and raise grievances, and does the school verify that the request comes from the parent or guardian?</t>
+    <t>Can students, or the parents of students under 18, ask to see, correct or erase the data and raise grievances, and does the institution verify who is asking?</t>
   </si>
   <si>
     <t>S.11-S.13, Rule 14</t>
   </si>
   <si>
-    <t xml:space="preserve">Rights request form or channel for parents
+    <t xml:space="preserve">Rights request form or channel for students and parents
 Requester verification procedure
 Rights and grievance request log</t>
   </si>
@@ -1240,7 +1240,7 @@
     <t>B12.13</t>
   </si>
   <si>
-    <t>Are student accounts on learning platforms and school apps set up without behavioural profiling or targeted advertising, and are the vendor terms checked for this?</t>
+    <t>Are student accounts on learning platforms and institution apps set up without behavioural profiling or targeted advertising of students under 18, and are the vendor terms checked for this?</t>
   </si>
   <si>
     <t>S.9(3), S.8(2)</t>

</xml_diff>